<commit_message>
data(p2p): refresh AP AR 2023-26 workbook and embedded copy
Ten rows changed against the deployed workbook, all fills of previously
blank or zero cells — no rows added, removed or reordered (461 non-empty
rows before and after, same single sheet, same header):

  G041 service providers — Results (Continued)/Net Achievement now
  populated for Kenya cooperatives (84) and five Tanzania stakeholder
  types (182, 186, 3, 4, 7).
  G051 direct jobs — Targets (Continued) now set for the four Tanzania
  worker segments (26950, 5145, 14700, 2205).

data-embedded.js is regenerated from the same byte snapshot as the
committed .xlsx (sha256 3cc4ede5…), so the fetch path and the file://
fallback serve identical data.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/masp4-platform/public/p2p/AP AR 2023-26.xlsx
+++ b/masp4-platform/public/p2p/AP AR 2023-26.xlsx
@@ -2334,10 +2334,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="4">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="I28" s="4">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="J28" s="4"/>
       <c r="K28" s="4">
@@ -7487,7 +7487,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="149" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" s="3" t="s">
         <v>56</v>
       </c>
@@ -7617,7 +7617,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="152" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" s="3" t="s">
         <v>56</v>
       </c>
@@ -7745,7 +7745,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="155" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" s="3" t="s">
         <v>56</v>
       </c>
@@ -11892,10 +11892,10 @@
         <v>0</v>
       </c>
       <c r="H255" s="4">
-        <v>0</v>
+        <v>182</v>
       </c>
       <c r="I255" s="4">
-        <v>0</v>
+        <v>182</v>
       </c>
       <c r="J255" s="4">
         <v>7</v>
@@ -12019,13 +12019,13 @@
         <v>23</v>
       </c>
       <c r="G258" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H258" s="4">
-        <v>0</v>
+        <v>181</v>
       </c>
       <c r="I258" s="4">
-        <v>0</v>
+        <v>186</v>
       </c>
       <c r="J258" s="4">
         <v>109</v>
@@ -12152,10 +12152,10 @@
         <v>0</v>
       </c>
       <c r="H261" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I261" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J261" s="4"/>
       <c r="K261" s="4">
@@ -12236,10 +12236,10 @@
         <v>0</v>
       </c>
       <c r="H263" s="4">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I263" s="4">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J263" s="4"/>
       <c r="K263" s="4">
@@ -12320,10 +12320,10 @@
         <v>0</v>
       </c>
       <c r="H265" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I265" s="4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J265" s="4">
         <v>14</v>
@@ -16851,7 +16851,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="372" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A372" s="3" t="s">
         <v>56</v>
       </c>
@@ -16981,7 +16981,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="375" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A375" s="3" t="s">
         <v>56</v>
       </c>
@@ -17629,7 +17629,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="390" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="390" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A390" s="3" t="s">
         <v>56</v>
       </c>
@@ -18845,7 +18845,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="418" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="418" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A418" s="3" t="s">
         <v>60</v>
       </c>
@@ -18887,7 +18887,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="419" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A419" s="3" t="s">
         <v>60</v>
       </c>
@@ -18916,7 +18916,9 @@
         <v>0</v>
       </c>
       <c r="J419" s="4"/>
-      <c r="K419" s="4"/>
+      <c r="K419" s="4">
+        <v>26950</v>
+      </c>
       <c r="L419" s="4">
         <v>0</v>
       </c>
@@ -18927,7 +18929,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="420" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="420" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A420" s="3" t="s">
         <v>60</v>
       </c>
@@ -18969,7 +18971,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="421" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="421" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A421" s="3" t="s">
         <v>60</v>
       </c>
@@ -18998,7 +19000,9 @@
         <v>0</v>
       </c>
       <c r="J421" s="4"/>
-      <c r="K421" s="4"/>
+      <c r="K421" s="4">
+        <v>5145</v>
+      </c>
       <c r="L421" s="4">
         <v>0</v>
       </c>
@@ -19009,7 +19013,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="422" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="422" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A422" s="3" t="s">
         <v>60</v>
       </c>
@@ -19051,7 +19055,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="423" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="423" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A423" s="3" t="s">
         <v>60</v>
       </c>
@@ -19080,7 +19084,9 @@
         <v>0</v>
       </c>
       <c r="J423" s="4"/>
-      <c r="K423" s="4"/>
+      <c r="K423" s="4">
+        <v>14700</v>
+      </c>
       <c r="L423" s="4">
         <v>0</v>
       </c>
@@ -19091,7 +19097,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="424" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="424" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A424" s="3" t="s">
         <v>60</v>
       </c>
@@ -19133,7 +19139,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="425" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="425" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A425" s="3" t="s">
         <v>60</v>
       </c>
@@ -19162,7 +19168,9 @@
         <v>0</v>
       </c>
       <c r="J425" s="4"/>
-      <c r="K425" s="4"/>
+      <c r="K425" s="4">
+        <v>2205</v>
+      </c>
       <c r="L425" s="4">
         <v>0</v>
       </c>
@@ -20547,19 +20555,14 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:N461">
-    <filterColumn colId="2">
+    <filterColumn colId="1">
       <filters>
-        <filter val="Gold"/>
+        <filter val="# of direct jobs supported by targeted producers"/>
       </filters>
     </filterColumn>
-    <filterColumn colId="5">
+    <filterColumn colId="12">
       <filters>
-        <filter val="2026"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="13">
-      <filters>
-        <filter val="# of producers supported with knowledge and skills"/>
+        <filter val="Pathways to Prosperity - Tanzania"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
fix(p2p): set Net annual target on the four G051 Tanzania worker rows
The targets entered for the Tanzania direct-jobs segments landed in
Targets (Continued) only; Net annual target stayed 0. app.js reads
Net Achievement and Net annual target and never the New/Continued
columns, so those four entries were invisible on the dashboard.

Sets L419/L421/L423/L425 to 26950 / 5145 / 14700 / 2205, matching
Targets (New) + Targets (Continued) — the rule the other 456 rows
already follow, and which now holds on all 460.

Effect on the dashboard: G051 target 157,713 -> 206,713, so the direct
jobs card moves from 74% to 56% of target; programme total target
5,619,372 -> 5,668,372 and overall 37.4% -> 37.1%. No achievement
figure changes.

Edited surgically in xl/worksheets/sheet1.xml so all 11 other zip
entries stay byte-identical; data-embedded.js regenerated from the
same snapshot (sha256 13596fa3…).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/masp4-platform/public/p2p/AP AR 2023-26.xlsx
+++ b/masp4-platform/public/p2p/AP AR 2023-26.xlsx
@@ -18920,7 +18920,7 @@
         <v>26950</v>
       </c>
       <c r="L419" s="4">
-        <v>0</v>
+        <v>26950</v>
       </c>
       <c r="M419" s="3" t="s">
         <v>85</v>
@@ -19004,7 +19004,7 @@
         <v>5145</v>
       </c>
       <c r="L421" s="4">
-        <v>0</v>
+        <v>5145</v>
       </c>
       <c r="M421" s="3" t="s">
         <v>85</v>
@@ -19088,7 +19088,7 @@
         <v>14700</v>
       </c>
       <c r="L423" s="4">
-        <v>0</v>
+        <v>14700</v>
       </c>
       <c r="M423" s="3" t="s">
         <v>85</v>
@@ -19172,7 +19172,7 @@
         <v>2205</v>
       </c>
       <c r="L425" s="4">
-        <v>0</v>
+        <v>2205</v>
       </c>
       <c r="M425" s="3" t="s">
         <v>85</v>

</xml_diff>

<commit_message>
data(p2p): refresh workbook — S2.1 Kenya target entries
Four rows changed (58, 61, 64, 67 — S2.1 producer services, Kenya):
Targets (New) and Targets (Continued) each set to 30871 / 16839 /
5893 / 2525. Net annual target on those rows is still 0, so no figure
the dashboard renders changes: programme total stays 2,102,591 vs
5,668,372 (37.1%).

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/masp4-platform/public/p2p/AP AR 2023-26.xlsx
+++ b/masp4-platform/public/p2p/AP AR 2023-26.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930"/>
+    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930"/>
   </bookViews>
   <sheets>
     <sheet name="report1785760719801" sheetId="1" r:id="rId1"/>
@@ -1235,7 +1235,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>14</v>
       </c>
@@ -1365,7 +1365,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -1495,7 +1495,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>14</v>
       </c>
@@ -1625,7 +1625,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
@@ -1755,7 +1755,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>14</v>
       </c>
@@ -1885,7 +1885,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>14</v>
       </c>
@@ -2015,7 +2015,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>14</v>
       </c>
@@ -2141,7 +2141,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>14</v>
       </c>
@@ -3323,7 +3323,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
         <v>41</v>
       </c>
@@ -3453,7 +3453,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="55" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
         <v>41</v>
       </c>
@@ -3581,7 +3581,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
         <v>43</v>
       </c>
@@ -3609,8 +3609,12 @@
       <c r="I58" s="4">
         <v>50302</v>
       </c>
-      <c r="J58" s="4"/>
-      <c r="K58" s="4"/>
+      <c r="J58" s="4">
+        <v>30871</v>
+      </c>
+      <c r="K58" s="4">
+        <v>30871</v>
+      </c>
       <c r="L58" s="4">
         <v>0</v>
       </c>
@@ -3705,7 +3709,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="61" spans="1:14" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
         <v>43</v>
       </c>
@@ -3733,8 +3737,12 @@
       <c r="I61" s="4">
         <v>18252</v>
       </c>
-      <c r="J61" s="4"/>
-      <c r="K61" s="4"/>
+      <c r="J61" s="4">
+        <v>16839</v>
+      </c>
+      <c r="K61" s="4">
+        <v>16839</v>
+      </c>
       <c r="L61" s="4">
         <v>0</v>
       </c>
@@ -3829,7 +3837,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="64" spans="1:14" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
         <v>43</v>
       </c>
@@ -3857,8 +3865,12 @@
       <c r="I64" s="4">
         <v>31215</v>
       </c>
-      <c r="J64" s="4"/>
-      <c r="K64" s="4"/>
+      <c r="J64" s="4">
+        <v>5893</v>
+      </c>
+      <c r="K64" s="4">
+        <v>5893</v>
+      </c>
       <c r="L64" s="4">
         <v>0</v>
       </c>
@@ -3953,7 +3965,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="67" spans="1:14" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A67" s="3" t="s">
         <v>43</v>
       </c>
@@ -3981,8 +3993,12 @@
       <c r="I67" s="4">
         <v>7936</v>
       </c>
-      <c r="J67" s="4"/>
-      <c r="K67" s="4"/>
+      <c r="J67" s="4">
+        <v>2525</v>
+      </c>
+      <c r="K67" s="4">
+        <v>2525</v>
+      </c>
       <c r="L67" s="4">
         <v>0</v>
       </c>
@@ -10791,7 +10807,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="230" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A230" s="3" t="s">
         <v>14</v>
       </c>
@@ -10921,7 +10937,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="233" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A233" s="3" t="s">
         <v>14</v>
       </c>
@@ -11051,7 +11067,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="236" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A236" s="3" t="s">
         <v>14</v>
       </c>
@@ -11181,7 +11197,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="239" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A239" s="3" t="s">
         <v>14</v>
       </c>
@@ -11311,7 +11327,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="242" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A242" s="3" t="s">
         <v>14</v>
       </c>
@@ -11441,7 +11457,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="245" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A245" s="3" t="s">
         <v>14</v>
       </c>
@@ -11571,7 +11587,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="248" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A248" s="3" t="s">
         <v>14</v>
       </c>
@@ -11699,7 +11715,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="251" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A251" s="3" t="s">
         <v>14</v>
       </c>
@@ -12883,7 +12899,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="279" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A279" s="3" t="s">
         <v>41</v>
       </c>
@@ -13013,7 +13029,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="282" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A282" s="3" t="s">
         <v>41</v>
       </c>
@@ -13263,7 +13279,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="288" spans="1:14" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A288" s="3" t="s">
         <v>43</v>
       </c>
@@ -13479,7 +13495,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="293" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A293" s="3" t="s">
         <v>41</v>
       </c>
@@ -13723,7 +13739,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="299" spans="1:14" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A299" s="3" t="s">
         <v>43</v>
       </c>
@@ -13889,7 +13905,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="303" spans="1:14" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A303" s="3" t="s">
         <v>43</v>
       </c>
@@ -14055,7 +14071,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="307" spans="1:14" ht="43.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A307" s="3" t="s">
         <v>43</v>
       </c>
@@ -18845,7 +18861,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="418" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="418" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A418" s="3" t="s">
         <v>60</v>
       </c>
@@ -18887,7 +18903,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="419" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="419" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A419" s="3" t="s">
         <v>60</v>
       </c>
@@ -18929,7 +18945,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="420" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="420" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A420" s="3" t="s">
         <v>60</v>
       </c>
@@ -18971,7 +18987,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="421" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="421" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A421" s="3" t="s">
         <v>60</v>
       </c>
@@ -19013,7 +19029,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="422" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="422" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A422" s="3" t="s">
         <v>60</v>
       </c>
@@ -19055,7 +19071,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="423" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="423" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A423" s="3" t="s">
         <v>60</v>
       </c>
@@ -19097,7 +19113,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="424" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="424" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A424" s="3" t="s">
         <v>60</v>
       </c>
@@ -19139,7 +19155,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="425" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="425" spans="1:14" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A425" s="3" t="s">
         <v>60</v>
       </c>
@@ -20557,12 +20573,14 @@
   <autoFilter ref="A1:N461">
     <filterColumn colId="1">
       <filters>
-        <filter val="# of direct jobs supported by targeted producers"/>
+        <filter val="# of farmers that access new or improved services from service providers supported by Solidaridad"/>
+        <filter val="# producers with new or improved access to services"/>
+        <filter val="# targeted producers with new or improved access to markets"/>
       </filters>
     </filterColumn>
-    <filterColumn colId="12">
+    <filterColumn colId="5">
       <filters>
-        <filter val="Pathways to Prosperity - Tanzania"/>
+        <filter val="2025"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
fix(p2p): set Net annual target on the four S2.1 Kenya rows
Same defect as the G051 rows: the figures were entered in the Targets
columns but Net annual target stayed 0, and app.js reads only Net
annual target. Sets L58/L61/L64/L67 to 30871 / 16839 / 5893 / 2525.

The value is the single figure entered, not New + Continued: the same
number appears in both Targets columns and one of the two is a
duplicate keystroke, confirmed by the programme team. The duplicate
itself is left in place — which column holds the real figure is not
established — so these four rows still read New+Continued != Net.

Dashboard effect: S2.1 target 361,741 -> 417,069; programme total
5,668,372 -> 5,724,500 and overall 37.1% -> 36.7%. No achievement
figure changes.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/masp4-platform/public/p2p/AP AR 2023-26.xlsx
+++ b/masp4-platform/public/p2p/AP AR 2023-26.xlsx
@@ -3616,7 +3616,7 @@
         <v>30871</v>
       </c>
       <c r="L58" s="4">
-        <v>0</v>
+        <v>30871</v>
       </c>
       <c r="M58" s="3" t="s">
         <v>20</v>
@@ -3744,7 +3744,7 @@
         <v>16839</v>
       </c>
       <c r="L61" s="4">
-        <v>0</v>
+        <v>16839</v>
       </c>
       <c r="M61" s="3" t="s">
         <v>20</v>
@@ -3872,7 +3872,7 @@
         <v>5893</v>
       </c>
       <c r="L64" s="4">
-        <v>0</v>
+        <v>5893</v>
       </c>
       <c r="M64" s="3" t="s">
         <v>20</v>
@@ -4000,7 +4000,7 @@
         <v>2525</v>
       </c>
       <c r="L67" s="4">
-        <v>0</v>
+        <v>2525</v>
       </c>
       <c r="M67" s="3" t="s">
         <v>20</v>

</xml_diff>